<commit_message>
Added Thermostat and Washig Machine to improved GUI
</commit_message>
<xml_diff>
--- a/unit-sh/shsXl.xlsx
+++ b/unit-sh/shsXl.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2391" uniqueCount="622">
   <si>
     <t>TASK_ID</t>
   </si>
@@ -1210,6 +1210,678 @@
   </si>
   <si>
     <t>2025-08-24T23:31:06.973585571+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-25T21:54:51.225744139+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-25T21:54:51.226110710+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-25T21:54:51.276814711+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-25T21:54:51.276926250+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-25T23:25:17.999308608+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-25T23:25:17.999532877+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-25T23:25:18.032623774+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-25T23:25:18.032740432+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T11:38:21.468125316+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T11:38:21.468494577+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T11:52:09.742851493+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T11:52:09.743126795+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T11:52:11.882507587+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T11:52:11.882904197+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T11:52:49.098776790+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T11:52:49.099143540+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T11:54:05.379423291+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T11:54:05.379601270+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T12:01:43.875883649+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T12:01:43.876314087+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T12:01:46.505882830+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T12:01:46.506412181+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T12:01:51.636197242+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T12:01:51.636690595+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T12:01:56.397929388+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T12:01:56.398182387+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T19:33:27.422700310+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T19:33:27.422950745+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T19:34:05.456560280+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T19:34:05.456685060+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:17.763660002+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:17.763859551+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:18.164483389+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:18.164580870+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:18.571556416+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:18.571643091+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:18.893488414+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:18.893577754+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:19.184539856+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:19.184597601+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:19.560921417+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:19.561127491+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:19.934276192+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:19.934365060+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:20.182307370+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:20.182378029+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:20.658183499+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:20.658413501+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:20.978693800+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:20.978751163+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:21.207216315+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:21.207270535+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:23.019148447+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:23.019230268+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:23.263796982+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:23.263876466+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:23.532723011+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:23.532784250+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:24.465246815+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:24.465372806+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:24.489895658+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:24.489947622+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:34.942993050+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:34.943060049+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:35.157060735+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:35.157109844+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:35.384213635+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:35.384264268+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:36.416779015+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:36.416904696+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:36.639274719+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:36.639320611+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:36.869270542+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:36.869322737+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:37.111361203+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:37.111409628+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:37.328610467+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:37.328652165+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:37.560877+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:37.560925294+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:37.782599392+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:37.782661278+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:37.994395732+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:37.994495772+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:38.241815658+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:38.241872863+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:38.555150429+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:38.555203232+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:38.774387667+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:38.774445731+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:39.000520057+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:39.000638474+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:39.350874907+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:39.350992494+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:39.554724706+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:39.554781337+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:39.758585626+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:39.758628813+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:41.182285239+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:41.182332810+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:41.403333795+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:41.403381822+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:41.642208945+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:41.642284518+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:41.943468239+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:41.943582088+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:44.510618231+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:44.510723431+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:44.726758714+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:44.726801617+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:45.087410510+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:45.087536867+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:46.430834615+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:46.430886118+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:46.645433844+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:46.645476173+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:48.271847696+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:48.271942111+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:48.499942992+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:48.500001878+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:48.701086275+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:48.701125364+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:48.921447266+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:48.921487045+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:49.368604083+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:49.368706415+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:49.494487905+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:49.494527729+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:49.703321122+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:20:49.703359999+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:22:28.282211277+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:22:28.282305643+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:23:21.525487291+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:23:21.525638386+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:23:26.552253938+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:23:26.552293628+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:23:42.658141162+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-08-26T20:23:42.658237010+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-01T18:34:28.575799564+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-01T18:34:28.576036770+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-01T18:34:51.109566648+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-01T18:34:51.109672427+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-01T21:43:05.043671067+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-01T21:43:05.043847094+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-01T21:43:28.349633448+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-01T21:43:28.349806752+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T08:54:06.303870998+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T08:54:06.304083377+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T08:54:10.236142530+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T08:54:10.236251219+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T08:54:14.353137120+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T08:54:14.353325230+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T10:10:33.112108677+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T10:10:33.112204421+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T10:20:21.070806646+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T10:20:21.071102856+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T10:21:16.063128383+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T10:21:16.063387419+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T10:23:23.021902735+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T10:23:23.022090743+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T10:23:24.589884857+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T10:23:24.590176740+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T10:23:29.619684793+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T10:23:29.619779962+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T10:23:37.686871982+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-02T10:23:37.686994521+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:24:24.074838661+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:24:24.075013117+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:24:24.098072103+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:24:24.098127270+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:24:47.196458003+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:24:47.196530080+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:24:52.236251321+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:24:52.236380255+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:25:25.223980934+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:25:25.224060141+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:25:25.547550361+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:25:25.547653416+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:25:25.898638065+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:25:25.898688315+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:25:26.227999485+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T09:25:26.228098419+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T15:25:31.776711060+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T15:25:31.778467904+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T15:25:33.016894057+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T15:25:33.017053483+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:13.390243926+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:13.390422508+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:13.943734073+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:13.943841246+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:14.529377771+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:14.529533289+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:17.392222658+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:17.392302160+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:17.894618653+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:17.894701317+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:18.345870953+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:18.345944159+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:21.525832419+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:21.525942240+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:22.007973414+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:22.008111050+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:22.453070749+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:22.453249390+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:22.897626898+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:22.897729497+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:23.327821495+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:23.327959852+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:23.780754876+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:23.780870356+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:24.241774609+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:24.241853695+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:24.762740753+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:15:24.762829282+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:27:55.337402971+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:27:55.337624104+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:27:55.972200472+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:27:55.972548868+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:27:56.669599668+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:27:56.669669145+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:30:01.121996070+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:30:01.122181635+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:30:01.173602576+02:00[Europe/Amsterdam]</t>
+  </si>
+  <si>
+    <t>2025-09-03T16:30:01.173882030+02:00[Europe/Amsterdam]</t>
   </si>
 </sst>
 </file>
@@ -1360,13 +2032,13 @@
         <v>109</v>
       </c>
       <c r="J2" t="s" s="0">
-        <v>64</v>
+        <v>111</v>
       </c>
       <c r="K2" t="s" s="0">
-        <v>183</v>
+        <v>400</v>
       </c>
       <c r="L2" t="s" s="0">
-        <v>184</v>
+        <v>401</v>
       </c>
       <c r="M2" t="s" s="0">
         <v>109</v>
@@ -1398,19 +2070,19 @@
         <v>1024.0</v>
       </c>
       <c r="I3" t="s" s="0">
-        <v>63</v>
+        <v>109</v>
       </c>
       <c r="J3" t="s" s="0">
-        <v>64</v>
+        <v>111</v>
       </c>
       <c r="K3" t="s" s="0">
-        <v>69</v>
+        <v>620</v>
       </c>
       <c r="L3" t="s" s="0">
-        <v>70</v>
+        <v>621</v>
       </c>
       <c r="M3" t="s" s="0">
-        <v>39</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4">
@@ -1480,19 +2152,19 @@
         <v>1024.0</v>
       </c>
       <c r="I5" t="s" s="0">
-        <v>63</v>
+        <v>109</v>
       </c>
       <c r="J5" t="s" s="0">
         <v>64</v>
       </c>
       <c r="K5" t="s" s="0">
-        <v>77</v>
+        <v>570</v>
       </c>
       <c r="L5" t="s" s="0">
-        <v>78</v>
+        <v>571</v>
       </c>
       <c r="M5" t="s" s="0">
-        <v>39</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6">
@@ -1644,19 +2316,19 @@
         <v>1024.0</v>
       </c>
       <c r="I9" t="s" s="0">
-        <v>63</v>
+        <v>109</v>
       </c>
       <c r="J9" t="s" s="0">
-        <v>64</v>
+        <v>111</v>
       </c>
       <c r="K9" t="s" s="0">
-        <v>92</v>
+        <v>566</v>
       </c>
       <c r="L9" t="s" s="0">
-        <v>93</v>
+        <v>567</v>
       </c>
       <c r="M9" t="s" s="0">
-        <v>39</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10">
@@ -1814,10 +2486,10 @@
         <v>111</v>
       </c>
       <c r="K13" t="s" s="0">
-        <v>322</v>
+        <v>616</v>
       </c>
       <c r="L13" t="s" s="0">
-        <v>323</v>
+        <v>617</v>
       </c>
       <c r="M13" t="s" s="0">
         <v>109</v>
@@ -1937,10 +2609,10 @@
         <v>64</v>
       </c>
       <c r="K16" t="s" s="0">
-        <v>326</v>
+        <v>578</v>
       </c>
       <c r="L16" t="s" s="0">
-        <v>327</v>
+        <v>579</v>
       </c>
       <c r="M16" t="s" s="0">
         <v>109</v>
@@ -2057,13 +2729,13 @@
         <v>109</v>
       </c>
       <c r="J19" t="s" s="0">
-        <v>111</v>
+        <v>64</v>
       </c>
       <c r="K19" t="s" s="0">
-        <v>366</v>
+        <v>404</v>
       </c>
       <c r="L19" t="s" s="0">
-        <v>367</v>
+        <v>405</v>
       </c>
       <c r="M19" t="s" s="0">
         <v>109</v>
@@ -2221,13 +2893,13 @@
         <v>109</v>
       </c>
       <c r="J23" t="s" s="0">
-        <v>64</v>
+        <v>111</v>
       </c>
       <c r="K23" t="s" s="0">
-        <v>334</v>
+        <v>526</v>
       </c>
       <c r="L23" t="s" s="0">
-        <v>335</v>
+        <v>527</v>
       </c>
       <c r="M23" t="s" s="0">
         <v>109</v>
@@ -2303,13 +2975,13 @@
         <v>109</v>
       </c>
       <c r="J25" t="s" s="0">
-        <v>64</v>
+        <v>111</v>
       </c>
       <c r="K25" t="s" s="0">
-        <v>368</v>
+        <v>582</v>
       </c>
       <c r="L25" t="s" s="0">
-        <v>369</v>
+        <v>583</v>
       </c>
       <c r="M25" t="s" s="0">
         <v>109</v>

</xml_diff>